<commit_message>
Update birthday test date
</commit_message>
<xml_diff>
--- a/data/birthdays.xlsx
+++ b/data/birthdays.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amitkumar/Downloads/github-actions-birthday-slack/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03F109B3-4606-2745-8DC5-C2FD325D3463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030DB31F-7338-4442-87ED-32BBE6A6B0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="600" windowWidth="18200" windowHeight="8500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10600" yWindow="3560" windowWidth="18200" windowHeight="8500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Birthdays" sheetId="1" r:id="rId1"/>
@@ -82,9 +82,6 @@
     <t>1997-12-25</t>
   </si>
   <si>
-    <t>U0678901234</t>
-  </si>
-  <si>
     <t>Vikas</t>
   </si>
   <si>
@@ -109,10 +106,13 @@
     <t>1996-03-12</t>
   </si>
   <si>
-    <t>U0901234567</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 1997-09-2</t>
+  </si>
+  <si>
+    <t>U09012345675</t>
+  </si>
+  <si>
+    <t>U067890123422</t>
   </si>
 </sst>
 </file>
@@ -511,7 +511,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -522,7 +522,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -580,37 +580,37 @@
         <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" t="s">
         <v>22</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" t="s">
         <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>29</v>

</xml_diff>